<commit_message>
att pedido 019 fertilidade
</commit_message>
<xml_diff>
--- a/pedidos/F2026019S.xlsx
+++ b/pedidos/F2026019S.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Agroserver\gestao_projetos\08_Processo_Químico\02_Clientes\OS_2026\ATVOS\OS_019\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agroroboticafca-my.sharepoint.com/personal/miguel_santos_agrorobotica_com_br/Documents/AGROROBOTICA/PROJETOS/Dashoboard_ATVOS/pedidos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE5D5708-9E8C-4ECF-AE42-96512AB6AABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{BE5D5708-9E8C-4ECF-AE42-96512AB6AABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5773366B-3384-4ABC-929A-824032DDEDD0}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>

<commit_message>
att 018 e 019
</commit_message>
<xml_diff>
--- a/pedidos/F2026019S.xlsx
+++ b/pedidos/F2026019S.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agroroboticafca-my.sharepoint.com/personal/miguel_santos_agrorobotica_com_br/Documents/AGROROBOTICA/PROJETOS/Dashoboard_ATVOS/pedidos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{BE5D5708-9E8C-4ECF-AE42-96512AB6AABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5D11494-A74D-4C7D-8AF7-0F238E0A38FC}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{BE5D5708-9E8C-4ECF-AE42-96512AB6AABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8C12DBE-36A5-4762-8204-9FD97869A56D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1562" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1684" uniqueCount="264">
   <si>
     <t>Obj-ID</t>
   </si>
@@ -792,6 +792,42 @@
   </si>
   <si>
     <t>X</t>
+  </si>
+  <si>
+    <t>FAZ. FLORES E M. ALTO LD. CAP. E RETIRINHO</t>
+  </si>
+  <si>
+    <t>FAZENDA VAUZINHO</t>
+  </si>
+  <si>
+    <t>FAZENDA RIO VERDE T. BARRAS, LD ALEGRE E SUCURIZINHO</t>
+  </si>
+  <si>
+    <t>FAZENDA RIO VERDE, LD: NOVO HORIZONTE III</t>
+  </si>
+  <si>
+    <t>FAZENDA BOA ESPERANÇA</t>
+  </si>
+  <si>
+    <t>FAZENDA MARANATA, LD: RIO VERDE</t>
+  </si>
+  <si>
+    <t>FAZENDA RIO VERDE, LD: PARAISO</t>
+  </si>
+  <si>
+    <t>FAZENDA RIO VERDE, LD: JAMEC</t>
+  </si>
+  <si>
+    <t>FAZENDA ESTÂNCIA ADRIANE</t>
+  </si>
+  <si>
+    <t>FAZENDA RIO VERDE, LD: OURO VERDE E FURNA</t>
+  </si>
+  <si>
+    <t>FAZENDA GALHEIROS</t>
+  </si>
+  <si>
+    <t>FAZENDA TRÊS BARRAS, LD: ÁGUA LIMPA, BUGRE</t>
   </si>
 </sst>
 </file>
@@ -1177,7 +1213,7 @@
     <col min="11" max="11" width="18.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="54" style="2" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="10.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="11.42578125" style="2" bestFit="1" customWidth="1"/>
@@ -1450,6 +1486,9 @@
       <c r="M2" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N2" s="2" t="s">
+        <v>252</v>
+      </c>
       <c r="O2" s="2">
         <v>440335</v>
       </c>
@@ -1530,6 +1569,9 @@
       <c r="M3" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N3" s="2" t="s">
+        <v>252</v>
+      </c>
       <c r="O3" s="2">
         <v>440335</v>
       </c>
@@ -1610,6 +1652,9 @@
       <c r="M4" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N4" s="2" t="s">
+        <v>252</v>
+      </c>
       <c r="O4" s="2">
         <v>440335</v>
       </c>
@@ -1689,6 +1734,9 @@
       </c>
       <c r="M5" s="2" t="s">
         <v>125</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>252</v>
       </c>
       <c r="O5" s="2">
         <v>440335</v>
@@ -1767,6 +1815,9 @@
       <c r="M6" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N6" s="2" t="s">
+        <v>252</v>
+      </c>
       <c r="O6" s="2">
         <v>440335</v>
       </c>
@@ -1844,6 +1895,9 @@
       <c r="M7" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N7" s="2" t="s">
+        <v>252</v>
+      </c>
       <c r="O7" s="2">
         <v>440335</v>
       </c>
@@ -1921,6 +1975,9 @@
       <c r="M8" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N8" s="2" t="s">
+        <v>252</v>
+      </c>
       <c r="O8" s="2">
         <v>440335</v>
       </c>
@@ -1998,6 +2055,9 @@
       <c r="M9" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N9" s="2" t="s">
+        <v>252</v>
+      </c>
       <c r="O9" s="2">
         <v>440335</v>
       </c>
@@ -2075,6 +2135,9 @@
       <c r="M10" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N10" s="2" t="s">
+        <v>253</v>
+      </c>
       <c r="O10" s="2">
         <v>440354</v>
       </c>
@@ -2155,6 +2218,9 @@
       <c r="M11" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N11" s="2" t="s">
+        <v>253</v>
+      </c>
       <c r="O11" s="2">
         <v>440354</v>
       </c>
@@ -2235,6 +2301,9 @@
       <c r="M12" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N12" s="2" t="s">
+        <v>253</v>
+      </c>
       <c r="O12" s="2">
         <v>440354</v>
       </c>
@@ -2315,6 +2384,9 @@
       <c r="M13" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N13" s="2" t="s">
+        <v>253</v>
+      </c>
       <c r="O13" s="2">
         <v>440354</v>
       </c>
@@ -2392,6 +2464,9 @@
       <c r="M14" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N14" s="2" t="s">
+        <v>253</v>
+      </c>
       <c r="O14" s="2">
         <v>440354</v>
       </c>
@@ -2469,6 +2544,9 @@
       <c r="M15" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N15" s="2" t="s">
+        <v>253</v>
+      </c>
       <c r="O15" s="2">
         <v>440354</v>
       </c>
@@ -2546,6 +2624,9 @@
       <c r="M16" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N16" s="2" t="s">
+        <v>253</v>
+      </c>
       <c r="O16" s="2">
         <v>440354</v>
       </c>
@@ -2623,6 +2704,9 @@
       <c r="M17" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N17" s="2" t="s">
+        <v>253</v>
+      </c>
       <c r="O17" s="2">
         <v>440354</v>
       </c>
@@ -2700,6 +2784,9 @@
       <c r="M18" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N18" s="2" t="s">
+        <v>253</v>
+      </c>
       <c r="O18" s="2">
         <v>440354</v>
       </c>
@@ -2780,6 +2867,9 @@
       <c r="M19" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N19" s="2" t="s">
+        <v>253</v>
+      </c>
       <c r="O19" s="2">
         <v>440354</v>
       </c>
@@ -2857,6 +2947,9 @@
       <c r="M20" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N20" s="2" t="s">
+        <v>253</v>
+      </c>
       <c r="O20" s="2">
         <v>440354</v>
       </c>
@@ -2934,6 +3027,9 @@
       <c r="M21" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N21" s="2" t="s">
+        <v>253</v>
+      </c>
       <c r="O21" s="2">
         <v>440354</v>
       </c>
@@ -3011,6 +3107,9 @@
       <c r="M22" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N22" s="2" t="s">
+        <v>253</v>
+      </c>
       <c r="O22" s="2">
         <v>440354</v>
       </c>
@@ -3088,6 +3187,9 @@
       <c r="M23" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N23" s="2" t="s">
+        <v>253</v>
+      </c>
       <c r="O23" s="2">
         <v>440354</v>
       </c>
@@ -3165,6 +3267,9 @@
       <c r="M24" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N24" s="2" t="s">
+        <v>253</v>
+      </c>
       <c r="O24" s="2">
         <v>440354</v>
       </c>
@@ -3242,6 +3347,9 @@
       <c r="M25" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N25" s="2" t="s">
+        <v>253</v>
+      </c>
       <c r="O25" s="2">
         <v>440354</v>
       </c>
@@ -3319,6 +3427,9 @@
       <c r="M26" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N26" s="2" t="s">
+        <v>253</v>
+      </c>
       <c r="O26" s="2">
         <v>440354</v>
       </c>
@@ -3396,6 +3507,9 @@
       <c r="M27" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N27" s="2" t="s">
+        <v>253</v>
+      </c>
       <c r="O27" s="2">
         <v>440354</v>
       </c>
@@ -3473,6 +3587,9 @@
       <c r="M28" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N28" s="2" t="s">
+        <v>254</v>
+      </c>
       <c r="O28" s="2">
         <v>440320</v>
       </c>
@@ -3553,6 +3670,9 @@
       <c r="M29" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N29" s="2" t="s">
+        <v>254</v>
+      </c>
       <c r="O29" s="2">
         <v>440320</v>
       </c>
@@ -3633,6 +3753,9 @@
       <c r="M30" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N30" s="2" t="s">
+        <v>255</v>
+      </c>
       <c r="O30" s="2">
         <v>440069</v>
       </c>
@@ -3713,6 +3836,9 @@
       <c r="M31" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N31" s="2" t="s">
+        <v>255</v>
+      </c>
       <c r="O31" s="2">
         <v>440069</v>
       </c>
@@ -3793,6 +3919,9 @@
       <c r="M32" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N32" s="2" t="s">
+        <v>256</v>
+      </c>
       <c r="O32" s="2">
         <v>440076</v>
       </c>
@@ -3873,6 +4002,9 @@
       <c r="M33" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N33" s="2" t="s">
+        <v>256</v>
+      </c>
       <c r="O33" s="2">
         <v>440076</v>
       </c>
@@ -3953,6 +4085,9 @@
       <c r="M34" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N34" s="2" t="s">
+        <v>256</v>
+      </c>
       <c r="O34" s="2">
         <v>440076</v>
       </c>
@@ -4033,6 +4168,9 @@
       <c r="M35" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N35" s="2" t="s">
+        <v>256</v>
+      </c>
       <c r="O35" s="2">
         <v>440076</v>
       </c>
@@ -4110,6 +4248,9 @@
       <c r="M36" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N36" s="2" t="s">
+        <v>256</v>
+      </c>
       <c r="O36" s="2">
         <v>440076</v>
       </c>
@@ -4187,6 +4328,9 @@
       <c r="M37" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N37" s="2" t="s">
+        <v>256</v>
+      </c>
       <c r="O37" s="2">
         <v>440076</v>
       </c>
@@ -4264,6 +4408,9 @@
       <c r="M38" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N38" s="2" t="s">
+        <v>257</v>
+      </c>
       <c r="O38" s="2">
         <v>440043</v>
       </c>
@@ -4344,6 +4491,9 @@
       <c r="M39" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N39" s="2" t="s">
+        <v>257</v>
+      </c>
       <c r="O39" s="2">
         <v>440043</v>
       </c>
@@ -4424,6 +4574,9 @@
       <c r="M40" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N40" s="2" t="s">
+        <v>257</v>
+      </c>
       <c r="O40" s="2">
         <v>440043</v>
       </c>
@@ -4504,6 +4657,9 @@
       <c r="M41" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N41" s="2" t="s">
+        <v>257</v>
+      </c>
       <c r="O41" s="2">
         <v>440043</v>
       </c>
@@ -4581,6 +4737,9 @@
       <c r="M42" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N42" s="2" t="s">
+        <v>257</v>
+      </c>
       <c r="O42" s="2">
         <v>440043</v>
       </c>
@@ -4658,6 +4817,9 @@
       <c r="M43" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N43" s="2" t="s">
+        <v>257</v>
+      </c>
       <c r="O43" s="2">
         <v>440043</v>
       </c>
@@ -4735,6 +4897,9 @@
       <c r="M44" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N44" s="2" t="s">
+        <v>257</v>
+      </c>
       <c r="O44" s="2">
         <v>440043</v>
       </c>
@@ -4812,6 +4977,9 @@
       <c r="M45" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N45" s="2" t="s">
+        <v>257</v>
+      </c>
       <c r="O45" s="2">
         <v>440043</v>
       </c>
@@ -4889,6 +5057,9 @@
       <c r="M46" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N46" s="2" t="s">
+        <v>257</v>
+      </c>
       <c r="O46" s="2">
         <v>440043</v>
       </c>
@@ -4966,6 +5137,9 @@
       <c r="M47" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N47" s="2" t="s">
+        <v>257</v>
+      </c>
       <c r="O47" s="2">
         <v>440043</v>
       </c>
@@ -5043,6 +5217,9 @@
       <c r="M48" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N48" s="2" t="s">
+        <v>257</v>
+      </c>
       <c r="O48" s="2">
         <v>440043</v>
       </c>
@@ -5123,6 +5300,9 @@
       <c r="M49" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N49" s="2" t="s">
+        <v>257</v>
+      </c>
       <c r="O49" s="2">
         <v>440043</v>
       </c>
@@ -5200,6 +5380,9 @@
       <c r="M50" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N50" s="2" t="s">
+        <v>257</v>
+      </c>
       <c r="O50" s="2">
         <v>440043</v>
       </c>
@@ -5277,6 +5460,9 @@
       <c r="M51" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N51" s="2" t="s">
+        <v>257</v>
+      </c>
       <c r="O51" s="2">
         <v>440043</v>
       </c>
@@ -5354,6 +5540,9 @@
       <c r="M52" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N52" s="2" t="s">
+        <v>258</v>
+      </c>
       <c r="O52" s="2">
         <v>440042</v>
       </c>
@@ -5434,6 +5623,9 @@
       <c r="M53" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N53" s="2" t="s">
+        <v>258</v>
+      </c>
       <c r="O53" s="2">
         <v>440042</v>
       </c>
@@ -5514,6 +5706,9 @@
       <c r="M54" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N54" s="2" t="s">
+        <v>258</v>
+      </c>
       <c r="O54" s="2">
         <v>440042</v>
       </c>
@@ -5594,6 +5789,9 @@
       <c r="M55" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N55" s="2" t="s">
+        <v>258</v>
+      </c>
       <c r="O55" s="2">
         <v>440042</v>
       </c>
@@ -5671,6 +5869,9 @@
       <c r="M56" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N56" s="2" t="s">
+        <v>258</v>
+      </c>
       <c r="O56" s="2">
         <v>440042</v>
       </c>
@@ -5748,6 +5949,9 @@
       <c r="M57" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N57" s="2" t="s">
+        <v>258</v>
+      </c>
       <c r="O57" s="2">
         <v>440042</v>
       </c>
@@ -5825,6 +6029,9 @@
       <c r="M58" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N58" s="2" t="s">
+        <v>258</v>
+      </c>
       <c r="O58" s="2">
         <v>440042</v>
       </c>
@@ -5902,6 +6109,9 @@
       <c r="M59" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N59" s="2" t="s">
+        <v>258</v>
+      </c>
       <c r="O59" s="2">
         <v>440042</v>
       </c>
@@ -5979,6 +6189,9 @@
       <c r="M60" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N60" s="2" t="s">
+        <v>258</v>
+      </c>
       <c r="O60" s="2">
         <v>440042</v>
       </c>
@@ -6056,6 +6269,9 @@
       <c r="M61" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N61" s="2" t="s">
+        <v>258</v>
+      </c>
       <c r="O61" s="2">
         <v>440042</v>
       </c>
@@ -6133,6 +6349,9 @@
       <c r="M62" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N62" s="2" t="s">
+        <v>258</v>
+      </c>
       <c r="O62" s="2">
         <v>440042</v>
       </c>
@@ -6210,6 +6429,9 @@
       <c r="M63" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N63" s="2" t="s">
+        <v>258</v>
+      </c>
       <c r="O63" s="2">
         <v>440042</v>
       </c>
@@ -6287,6 +6509,9 @@
       <c r="M64" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N64" s="2" t="s">
+        <v>259</v>
+      </c>
       <c r="O64" s="2">
         <v>440014</v>
       </c>
@@ -6367,6 +6592,9 @@
       <c r="M65" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N65" s="2" t="s">
+        <v>259</v>
+      </c>
       <c r="O65" s="2">
         <v>440014</v>
       </c>
@@ -6447,6 +6675,9 @@
       <c r="M66" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N66" s="2" t="s">
+        <v>259</v>
+      </c>
       <c r="O66" s="2">
         <v>440014</v>
       </c>
@@ -6524,6 +6755,9 @@
       <c r="M67" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N67" s="2" t="s">
+        <v>259</v>
+      </c>
       <c r="O67" s="2">
         <v>440014</v>
       </c>
@@ -6601,6 +6835,9 @@
       <c r="M68" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N68" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O68" s="2">
         <v>440031</v>
       </c>
@@ -6681,6 +6918,9 @@
       <c r="M69" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N69" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O69" s="2">
         <v>440031</v>
       </c>
@@ -6761,6 +7001,9 @@
       <c r="M70" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N70" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O70" s="2">
         <v>440031</v>
       </c>
@@ -6841,6 +7084,9 @@
       <c r="M71" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N71" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O71" s="2">
         <v>440031</v>
       </c>
@@ -6918,6 +7164,9 @@
       <c r="M72" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N72" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O72" s="2">
         <v>440031</v>
       </c>
@@ -6995,6 +7244,9 @@
       <c r="M73" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N73" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O73" s="2">
         <v>440031</v>
       </c>
@@ -7072,6 +7324,9 @@
       <c r="M74" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N74" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O74" s="2">
         <v>440031</v>
       </c>
@@ -7149,6 +7404,9 @@
       <c r="M75" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N75" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O75" s="2">
         <v>440031</v>
       </c>
@@ -7226,6 +7484,9 @@
       <c r="M76" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N76" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O76" s="2">
         <v>440031</v>
       </c>
@@ -7303,6 +7564,9 @@
       <c r="M77" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N77" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O77" s="2">
         <v>440031</v>
       </c>
@@ -7380,6 +7644,9 @@
       <c r="M78" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N78" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O78" s="2">
         <v>440031</v>
       </c>
@@ -7457,6 +7724,9 @@
       <c r="M79" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N79" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O79" s="2">
         <v>440031</v>
       </c>
@@ -7534,6 +7804,9 @@
       <c r="M80" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N80" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O80" s="2">
         <v>440031</v>
       </c>
@@ -7611,6 +7884,9 @@
       <c r="M81" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N81" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O81" s="2">
         <v>440031</v>
       </c>
@@ -7688,6 +7964,9 @@
       <c r="M82" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N82" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O82" s="2">
         <v>440031</v>
       </c>
@@ -7765,6 +8044,9 @@
       <c r="M83" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N83" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O83" s="2">
         <v>440031</v>
       </c>
@@ -7842,6 +8124,9 @@
       <c r="M84" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N84" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O84" s="2">
         <v>440031</v>
       </c>
@@ -7922,6 +8207,9 @@
       <c r="M85" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N85" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O85" s="2">
         <v>440031</v>
       </c>
@@ -7999,6 +8287,9 @@
       <c r="M86" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N86" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O86" s="2">
         <v>440031</v>
       </c>
@@ -8076,6 +8367,9 @@
       <c r="M87" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N87" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O87" s="2">
         <v>440031</v>
       </c>
@@ -8153,6 +8447,9 @@
       <c r="M88" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N88" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O88" s="2">
         <v>440031</v>
       </c>
@@ -8230,6 +8527,9 @@
       <c r="M89" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N89" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O89" s="2">
         <v>440031</v>
       </c>
@@ -8307,6 +8607,9 @@
       <c r="M90" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N90" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O90" s="2">
         <v>440031</v>
       </c>
@@ -8384,6 +8687,9 @@
       <c r="M91" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N91" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O91" s="2">
         <v>440031</v>
       </c>
@@ -8461,6 +8767,9 @@
       <c r="M92" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N92" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O92" s="2">
         <v>440031</v>
       </c>
@@ -8541,6 +8850,9 @@
       <c r="M93" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N93" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="O93" s="2">
         <v>440031</v>
       </c>
@@ -8618,6 +8930,9 @@
       <c r="M94" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N94" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="O94" s="2">
         <v>440118</v>
       </c>
@@ -8698,6 +9013,9 @@
       <c r="M95" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N95" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="O95" s="2">
         <v>440118</v>
       </c>
@@ -8778,6 +9096,9 @@
       <c r="M96" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N96" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="O96" s="2">
         <v>440118</v>
       </c>
@@ -8858,6 +9179,9 @@
       <c r="M97" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N97" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="O97" s="2">
         <v>440118</v>
       </c>
@@ -8935,6 +9259,9 @@
       <c r="M98" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N98" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="O98" s="2">
         <v>440118</v>
       </c>
@@ -9012,6 +9339,9 @@
       <c r="M99" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N99" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="O99" s="2">
         <v>440118</v>
       </c>
@@ -9089,6 +9419,9 @@
       <c r="M100" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N100" s="2" t="s">
+        <v>254</v>
+      </c>
       <c r="O100" s="2">
         <v>440320</v>
       </c>
@@ -9166,6 +9499,9 @@
       <c r="M101" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N101" s="2" t="s">
+        <v>254</v>
+      </c>
       <c r="O101" s="2">
         <v>440320</v>
       </c>
@@ -9243,6 +9579,9 @@
       <c r="M102" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N102" s="2" t="s">
+        <v>262</v>
+      </c>
       <c r="O102" s="2">
         <v>440049</v>
       </c>
@@ -9323,6 +9662,9 @@
       <c r="M103" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N103" s="2" t="s">
+        <v>262</v>
+      </c>
       <c r="O103" s="2">
         <v>440049</v>
       </c>
@@ -9403,6 +9745,9 @@
       <c r="M104" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N104" s="2" t="s">
+        <v>262</v>
+      </c>
       <c r="O104" s="2">
         <v>440049</v>
       </c>
@@ -9483,6 +9828,9 @@
       <c r="M105" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N105" s="2" t="s">
+        <v>262</v>
+      </c>
       <c r="O105" s="2">
         <v>440049</v>
       </c>
@@ -9560,6 +9908,9 @@
       <c r="M106" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N106" s="2" t="s">
+        <v>262</v>
+      </c>
       <c r="O106" s="2">
         <v>440049</v>
       </c>
@@ -9637,6 +9988,9 @@
       <c r="M107" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N107" s="2" t="s">
+        <v>262</v>
+      </c>
       <c r="O107" s="2">
         <v>440049</v>
       </c>
@@ -9714,6 +10068,9 @@
       <c r="M108" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N108" s="2" t="s">
+        <v>262</v>
+      </c>
       <c r="O108" s="2">
         <v>440049</v>
       </c>
@@ -9791,6 +10148,9 @@
       <c r="M109" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N109" s="2" t="s">
+        <v>262</v>
+      </c>
       <c r="O109" s="2">
         <v>440049</v>
       </c>
@@ -9868,6 +10228,9 @@
       <c r="M110" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N110" s="2" t="s">
+        <v>262</v>
+      </c>
       <c r="O110" s="2">
         <v>440049</v>
       </c>
@@ -9945,6 +10308,9 @@
       <c r="M111" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N111" s="2" t="s">
+        <v>262</v>
+      </c>
       <c r="O111" s="2">
         <v>440049</v>
       </c>
@@ -10022,6 +10388,9 @@
       <c r="M112" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N112" s="2" t="s">
+        <v>262</v>
+      </c>
       <c r="O112" s="2">
         <v>440049</v>
       </c>
@@ -10099,6 +10468,9 @@
       <c r="M113" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N113" s="2" t="s">
+        <v>262</v>
+      </c>
       <c r="O113" s="2">
         <v>440049</v>
       </c>
@@ -10176,6 +10548,9 @@
       <c r="M114" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N114" s="2" t="s">
+        <v>263</v>
+      </c>
       <c r="O114" s="2">
         <v>440078</v>
       </c>
@@ -10256,6 +10631,9 @@
       <c r="M115" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N115" s="2" t="s">
+        <v>263</v>
+      </c>
       <c r="O115" s="2">
         <v>440078</v>
       </c>
@@ -10336,6 +10714,9 @@
       <c r="M116" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N116" s="2" t="s">
+        <v>263</v>
+      </c>
       <c r="O116" s="2">
         <v>440078</v>
       </c>
@@ -10416,6 +10797,9 @@
       <c r="M117" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N117" s="2" t="s">
+        <v>263</v>
+      </c>
       <c r="O117" s="2">
         <v>440078</v>
       </c>
@@ -10493,6 +10877,9 @@
       <c r="M118" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N118" s="2" t="s">
+        <v>263</v>
+      </c>
       <c r="O118" s="2">
         <v>440078</v>
       </c>
@@ -10570,6 +10957,9 @@
       <c r="M119" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N119" s="2" t="s">
+        <v>263</v>
+      </c>
       <c r="O119" s="2">
         <v>440078</v>
       </c>
@@ -10647,6 +11037,9 @@
       <c r="M120" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N120" s="2" t="s">
+        <v>263</v>
+      </c>
       <c r="O120" s="2">
         <v>440078</v>
       </c>
@@ -10724,6 +11117,9 @@
       <c r="M121" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N121" s="2" t="s">
+        <v>263</v>
+      </c>
       <c r="O121" s="2">
         <v>440078</v>
       </c>
@@ -10801,6 +11197,9 @@
       <c r="M122" s="2" t="s">
         <v>125</v>
       </c>
+      <c r="N122" s="2" t="s">
+        <v>263</v>
+      </c>
       <c r="O122" s="2">
         <v>440078</v>
       </c>
@@ -10877,6 +11276,9 @@
       </c>
       <c r="M123" s="2" t="s">
         <v>125</v>
+      </c>
+      <c r="N123" s="2" t="s">
+        <v>263</v>
       </c>
       <c r="O123" s="2">
         <v>440078</v>

</xml_diff>

<commit_message>
att planilhas de entrada
</commit_message>
<xml_diff>
--- a/pedidos/F2026019S.xlsx
+++ b/pedidos/F2026019S.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agroroboticafca-my.sharepoint.com/personal/miguel_santos_agrorobotica_com_br/Documents/AGROROBOTICA/PROJETOS/Dashoboard_ATVOS/pedidos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{BE5D5708-9E8C-4ECF-AE42-96512AB6AABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8C12DBE-36A5-4762-8204-9FD97869A56D}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{BE5D5708-9E8C-4ECF-AE42-96512AB6AABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12427DAE-0477-478A-8D54-DEE97A06B576}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -909,6 +909,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>